<commit_message>
planilhas com dados fictícios
</commit_message>
<xml_diff>
--- a/planilhas/RESGATES A FAVOR DO GOVER 04_05_2026.xlsx
+++ b/planilhas/RESGATES A FAVOR DO GOVER 04_05_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sefazrj.sharepoint.com/sites/SUBTES/Shared Documents/SUPGO/COOGO/Arquivos DJO Banco do Brasil/2026/05 - Maio/Resgates a Favor do Governo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\cifs-zone1\tesouro\Programas da SUPCONC\Programa SEI\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_12D623E9001C25F5E52E733EB808C68D7A195D7F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A7BCBF0-537C-4D1B-AA53-7DDB729E424A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA79D342-2BCC-475D-BBA6-73229473B10D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESGATES A FAVOR DO GOVER" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="88">
   <si>
     <t>NUMERO_DO_PROCESSO</t>
   </si>
@@ -125,12 +125,6 @@
     <t>5º JUIZ.ESP.FAZ.PÚBLIC</t>
   </si>
   <si>
-    <t>BEATRIZ SALLES PEREIRA</t>
-  </si>
-  <si>
-    <t>ESTADO DO RIO DE JANEIRO</t>
-  </si>
-  <si>
     <t>0200127468247</t>
   </si>
   <si>
@@ -158,9 +152,6 @@
     <t>CENTRAL DA DIVIDA ATIVA</t>
   </si>
   <si>
-    <t>SONIA DE FATIMA DA SILVA GUEDE</t>
-  </si>
-  <si>
     <t>0300103576707</t>
   </si>
   <si>
@@ -179,9 +170,6 @@
     <t>17 VARA DA FAZENDA</t>
   </si>
   <si>
-    <t>ELZA COELHO PINHEIRO</t>
-  </si>
-  <si>
     <t>0300113316110</t>
   </si>
   <si>
@@ -194,12 +182,6 @@
     <t>8 NUCLEO 4.0 DIR FAZEN</t>
   </si>
   <si>
-    <t>SECRETARIA DE ESTADO DE FAZEND</t>
-  </si>
-  <si>
-    <t>SENCINET BRASIL SERVICOS DE TE</t>
-  </si>
-  <si>
     <t>0700131748013</t>
   </si>
   <si>
@@ -218,9 +200,6 @@
     <t>01148688020238190001</t>
   </si>
   <si>
-    <t>REIMO ARTIGOS ESPORTIVOS LTDA.</t>
-  </si>
-  <si>
     <t>1000115485022</t>
   </si>
   <si>
@@ -278,9 +257,6 @@
     <t>ORGAO ESPECIAL DO TJ</t>
   </si>
   <si>
-    <t>JOSE EDUARDO FIGUEIREDO BRAUNS</t>
-  </si>
-  <si>
     <t>1800107349994</t>
   </si>
   <si>
@@ -290,9 +266,6 @@
     <t>01063873120238190001</t>
   </si>
   <si>
-    <t>RODOVIARIO NOVA GRECIA TRANSPO</t>
-  </si>
-  <si>
     <t>2000131754244</t>
   </si>
   <si>
@@ -302,9 +275,6 @@
     <t>01262884820248190001</t>
   </si>
   <si>
-    <t>JANETE RODRIGUES COSME REIS</t>
-  </si>
-  <si>
     <t>2800106772762</t>
   </si>
   <si>
@@ -317,13 +287,19 @@
     <t>01135096120248190001</t>
   </si>
   <si>
-    <t>BORLA BIANCA FERDINANDA VINCEN</t>
-  </si>
-  <si>
     <t>2800109993584</t>
   </si>
   <si>
     <t>20250033729156</t>
+  </si>
+  <si>
+    <t>NOME OU EMPRESA</t>
+  </si>
+  <si>
+    <t>12345678910</t>
+  </si>
+  <si>
+    <t>12345678901234</t>
   </si>
 </sst>
 </file>
@@ -383,12 +359,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,6 +381,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -694,6 +675,7 @@
   <dimension ref="A1:Y30"/>
   <sheetFormatPr defaultColWidth="35" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="9" max="9" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="43.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -791,25 +773,25 @@
         <v>2234</v>
       </c>
       <c r="F2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J2" t="s">
         <v>29</v>
       </c>
-      <c r="G2">
-        <v>16572699730</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>30</v>
       </c>
-      <c r="I2">
-        <v>42498600000171</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>31</v>
-      </c>
-      <c r="K2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" t="s">
-        <v>33</v>
       </c>
       <c r="M2" s="2">
         <v>46009</v>
@@ -839,54 +821,54 @@
         <v>0</v>
       </c>
       <c r="V2" t="s">
+        <v>32</v>
+      </c>
+      <c r="W2" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" t="s">
         <v>34</v>
-      </c>
-      <c r="W2" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E3">
         <v>2234</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" t="s">
         <v>40</v>
-      </c>
-      <c r="I3">
-        <v>98750283715</v>
-      </c>
-      <c r="J3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3" t="s">
-        <v>43</v>
       </c>
       <c r="M3" s="2">
         <v>45538</v>
@@ -916,54 +898,54 @@
         <v>0</v>
       </c>
       <c r="V3" t="s">
+        <v>32</v>
+      </c>
+      <c r="W3" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y3" t="s">
         <v>34</v>
-      </c>
-      <c r="W3" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
         <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E4">
         <v>2234</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4">
-        <v>2101319772</v>
+        <v>85</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="J4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="M4" s="2">
         <v>45789</v>
@@ -993,54 +975,54 @@
         <v>0</v>
       </c>
       <c r="V4" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X4" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" t="s">
         <v>34</v>
-      </c>
-      <c r="W4" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X4" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
         <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>2234</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5">
-        <v>42498675000152</v>
+        <v>85</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5">
-        <v>33179565000137</v>
+        <v>85</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M5" s="2">
         <v>45351</v>
@@ -1070,54 +1052,54 @@
         <v>0</v>
       </c>
       <c r="V5" t="s">
+        <v>32</v>
+      </c>
+      <c r="W5" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y5" t="s">
         <v>34</v>
-      </c>
-      <c r="W5" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X5" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E6">
         <v>2234</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6">
-        <v>42498675000152</v>
+        <v>85</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6">
-        <v>33179565000137</v>
+        <v>85</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M6" s="2">
         <v>45351</v>
@@ -1147,54 +1129,54 @@
         <v>0</v>
       </c>
       <c r="V6" t="s">
+        <v>32</v>
+      </c>
+      <c r="W6" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X6" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y6" t="s">
         <v>34</v>
-      </c>
-      <c r="W6" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X6" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E7">
         <v>2234</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7">
-        <v>42498675000152</v>
+        <v>85</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7">
-        <v>33179565000137</v>
+        <v>85</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="L7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M7" s="2">
         <v>45351</v>
@@ -1224,54 +1206,54 @@
         <v>0</v>
       </c>
       <c r="V7" t="s">
+        <v>32</v>
+      </c>
+      <c r="W7" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y7" t="s">
         <v>34</v>
-      </c>
-      <c r="W7" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X7" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E8">
         <v>2234</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8">
-        <v>42498675000152</v>
+        <v>85</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8">
-        <v>33179565000137</v>
+        <v>85</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="L8" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M8" s="2">
         <v>45351</v>
@@ -1301,54 +1283,54 @@
         <v>0</v>
       </c>
       <c r="V8" t="s">
+        <v>32</v>
+      </c>
+      <c r="W8" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X8" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y8" t="s">
         <v>34</v>
-      </c>
-      <c r="W8" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X8" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E9">
         <v>2234</v>
       </c>
       <c r="F9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H9" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" t="s">
         <v>52</v>
       </c>
-      <c r="G9">
-        <v>42498675000152</v>
-      </c>
-      <c r="H9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9">
-        <v>33179565000137</v>
-      </c>
-      <c r="J9" t="s">
-        <v>54</v>
-      </c>
-      <c r="K9" t="s">
-        <v>58</v>
-      </c>
       <c r="L9" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M9" s="2">
         <v>45397</v>
@@ -1378,54 +1360,54 @@
         <v>0</v>
       </c>
       <c r="V9" t="s">
+        <v>32</v>
+      </c>
+      <c r="W9" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X9" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y9" t="s">
         <v>34</v>
-      </c>
-      <c r="W9" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X9" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E10">
         <v>2234</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
-      </c>
-      <c r="I10">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J10" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L10" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="M10" s="2">
         <v>45852</v>
@@ -1455,54 +1437,54 @@
         <v>0</v>
       </c>
       <c r="V10" t="s">
+        <v>32</v>
+      </c>
+      <c r="W10" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X10" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y10" t="s">
         <v>34</v>
-      </c>
-      <c r="W10" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X10" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E11">
         <v>2234</v>
       </c>
       <c r="F11" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" t="s">
+        <v>85</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K11" t="s">
         <v>30</v>
       </c>
-      <c r="G11">
-        <v>42498600000171</v>
-      </c>
-      <c r="H11" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11">
-        <v>1296286000167</v>
-      </c>
-      <c r="J11" t="s">
-        <v>61</v>
-      </c>
-      <c r="K11" t="s">
-        <v>32</v>
-      </c>
       <c r="L11" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="M11" s="2">
         <v>45852</v>
@@ -1532,54 +1514,54 @@
         <v>0</v>
       </c>
       <c r="V11" t="s">
+        <v>32</v>
+      </c>
+      <c r="W11" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X11" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y11" t="s">
         <v>34</v>
-      </c>
-      <c r="W11" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X11" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E12">
         <v>2234</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
-      </c>
-      <c r="I12">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J12" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K12" t="s">
+        <v>50</v>
+      </c>
+      <c r="L12" t="s">
         <v>56</v>
-      </c>
-      <c r="L12" t="s">
-        <v>63</v>
       </c>
       <c r="M12" s="2">
         <v>45852</v>
@@ -1609,54 +1591,54 @@
         <v>0</v>
       </c>
       <c r="V12" t="s">
+        <v>32</v>
+      </c>
+      <c r="W12" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X12" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y12" t="s">
         <v>34</v>
-      </c>
-      <c r="W12" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X12" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E13">
         <v>2234</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H13" t="s">
-        <v>60</v>
-      </c>
-      <c r="I13">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K13" t="s">
+        <v>51</v>
+      </c>
+      <c r="L13" t="s">
         <v>57</v>
-      </c>
-      <c r="L13" t="s">
-        <v>64</v>
       </c>
       <c r="M13" s="2">
         <v>45852</v>
@@ -1686,54 +1668,54 @@
         <v>0</v>
       </c>
       <c r="V13" t="s">
+        <v>32</v>
+      </c>
+      <c r="W13" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X13" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y13" t="s">
         <v>34</v>
-      </c>
-      <c r="W13" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X13" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E14">
         <v>2234</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H14" t="s">
-        <v>60</v>
-      </c>
-      <c r="I14">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J14" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K14" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L14" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="M14" s="2">
         <v>45852</v>
@@ -1763,54 +1745,54 @@
         <v>0</v>
       </c>
       <c r="V14" t="s">
+        <v>32</v>
+      </c>
+      <c r="W14" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y14" t="s">
         <v>34</v>
-      </c>
-      <c r="W14" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X14" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E15">
         <v>2234</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
-      </c>
-      <c r="G15">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
-      </c>
-      <c r="I15">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J15" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="L15" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="M15" s="2">
         <v>45852</v>
@@ -1840,54 +1822,54 @@
         <v>0</v>
       </c>
       <c r="V15" t="s">
+        <v>32</v>
+      </c>
+      <c r="W15" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X15" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y15" t="s">
         <v>34</v>
-      </c>
-      <c r="W15" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X15" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B16" t="s">
         <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E16">
         <v>2234</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
-      </c>
-      <c r="G16">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H16" t="s">
+        <v>85</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K16" t="s">
         <v>60</v>
       </c>
-      <c r="I16">
-        <v>1296286000167</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="L16" t="s">
         <v>61</v>
-      </c>
-      <c r="K16" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16" t="s">
-        <v>68</v>
       </c>
       <c r="M16" s="2">
         <v>45852</v>
@@ -1917,54 +1899,54 @@
         <v>0</v>
       </c>
       <c r="V16" t="s">
+        <v>32</v>
+      </c>
+      <c r="W16" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X16" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y16" t="s">
         <v>34</v>
-      </c>
-      <c r="W16" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X16" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
         <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E17">
         <v>2234</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
-      </c>
-      <c r="G17">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
-      </c>
-      <c r="I17">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J17" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L17" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="M17" s="2">
         <v>45852</v>
@@ -1994,54 +1976,54 @@
         <v>0</v>
       </c>
       <c r="V17" t="s">
+        <v>32</v>
+      </c>
+      <c r="W17" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X17" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y17" t="s">
         <v>34</v>
-      </c>
-      <c r="W17" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X17" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E18">
         <v>2234</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
-      </c>
-      <c r="G18">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H18" t="s">
-        <v>60</v>
-      </c>
-      <c r="I18">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J18" t="s">
+        <v>54</v>
+      </c>
+      <c r="K18" t="s">
+        <v>64</v>
+      </c>
+      <c r="L18" t="s">
         <v>61</v>
-      </c>
-      <c r="K18" t="s">
-        <v>71</v>
-      </c>
-      <c r="L18" t="s">
-        <v>68</v>
       </c>
       <c r="M18" s="2">
         <v>45852</v>
@@ -2071,54 +2053,54 @@
         <v>0</v>
       </c>
       <c r="V18" t="s">
+        <v>32</v>
+      </c>
+      <c r="W18" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X18" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y18" t="s">
         <v>34</v>
-      </c>
-      <c r="W18" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X18" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y18" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E19">
         <v>2234</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
-      </c>
-      <c r="G19">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H19" t="s">
-        <v>60</v>
-      </c>
-      <c r="I19">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J19" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="L19" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="M19" s="2">
         <v>45852</v>
@@ -2148,54 +2130,54 @@
         <v>0</v>
       </c>
       <c r="V19" t="s">
+        <v>32</v>
+      </c>
+      <c r="W19" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y19" t="s">
         <v>34</v>
-      </c>
-      <c r="W19" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X19" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y19" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
         <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E20">
         <v>2234</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
-      </c>
-      <c r="G20">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
-      </c>
-      <c r="I20">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J20" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K20" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="L20" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="M20" s="2">
         <v>45852</v>
@@ -2225,54 +2207,54 @@
         <v>0</v>
       </c>
       <c r="V20" t="s">
+        <v>32</v>
+      </c>
+      <c r="W20" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X20" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y20" t="s">
         <v>34</v>
-      </c>
-      <c r="W20" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X20" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
         <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E21">
         <v>2234</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H21" t="s">
-        <v>60</v>
-      </c>
-      <c r="I21">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J21" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K21" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="L21" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="M21" s="2">
         <v>45852</v>
@@ -2302,54 +2284,54 @@
         <v>0</v>
       </c>
       <c r="V21" t="s">
+        <v>32</v>
+      </c>
+      <c r="W21" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X21" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y21" t="s">
         <v>34</v>
-      </c>
-      <c r="W21" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X21" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E22">
         <v>2234</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
-      </c>
-      <c r="G22">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H22" t="s">
-        <v>60</v>
-      </c>
-      <c r="I22">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J22" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K22" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="L22" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="M22" s="2">
         <v>45852</v>
@@ -2379,54 +2361,54 @@
         <v>0</v>
       </c>
       <c r="V22" t="s">
+        <v>32</v>
+      </c>
+      <c r="W22" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y22" t="s">
         <v>34</v>
-      </c>
-      <c r="W22" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X22" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y22" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
         <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E23">
         <v>2234</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
-      </c>
-      <c r="G23">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H23" t="s">
-        <v>60</v>
-      </c>
-      <c r="I23">
-        <v>1296286000167</v>
+        <v>85</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J23" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="K23" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="L23" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="M23" s="2">
         <v>45852</v>
@@ -2456,54 +2438,54 @@
         <v>0</v>
       </c>
       <c r="V23" t="s">
+        <v>32</v>
+      </c>
+      <c r="W23" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X23" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y23" t="s">
         <v>34</v>
-      </c>
-      <c r="W23" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X23" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y23" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
         <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E24">
         <v>2234</v>
       </c>
       <c r="F24" t="s">
-        <v>80</v>
-      </c>
-      <c r="G24">
-        <v>76616274772</v>
+        <v>85</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="H24" t="s">
-        <v>30</v>
-      </c>
-      <c r="I24">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J24" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="K24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L24" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="M24" s="2">
         <v>45233</v>
@@ -2533,54 +2515,54 @@
         <v>0</v>
       </c>
       <c r="V24" t="s">
+        <v>32</v>
+      </c>
+      <c r="W24" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X24" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y24" t="s">
         <v>34</v>
-      </c>
-      <c r="W24" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X24" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y24" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
         <v>26</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E25">
         <v>2234</v>
       </c>
       <c r="F25" t="s">
-        <v>52</v>
-      </c>
-      <c r="G25">
-        <v>42498675000152</v>
+        <v>85</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H25" t="s">
-        <v>84</v>
-      </c>
-      <c r="I25">
-        <v>30263242000139</v>
+        <v>85</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="J25" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="K25" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L25" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="M25" s="2">
         <v>45351</v>
@@ -2610,54 +2592,54 @@
         <v>0</v>
       </c>
       <c r="V25" t="s">
+        <v>32</v>
+      </c>
+      <c r="W25" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X25" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y25" t="s">
         <v>34</v>
-      </c>
-      <c r="W25" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X25" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B26" t="s">
         <v>26</v>
       </c>
       <c r="C26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E26">
         <v>2234</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H26" t="s">
-        <v>88</v>
-      </c>
-      <c r="I26">
-        <v>52052192700</v>
+        <v>85</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="J26" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K26" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L26" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="M26" s="2">
         <v>45783</v>
@@ -2687,54 +2669,54 @@
         <v>0</v>
       </c>
       <c r="V26" t="s">
+        <v>32</v>
+      </c>
+      <c r="W26" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X26" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y26" t="s">
         <v>34</v>
-      </c>
-      <c r="W26" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X26" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y26" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B27" t="s">
         <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D27" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E27">
         <v>2234</v>
       </c>
       <c r="F27" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H27" t="s">
+        <v>85</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J27" t="s">
+        <v>79</v>
+      </c>
+      <c r="K27" t="s">
         <v>30</v>
       </c>
-      <c r="G27">
-        <v>42498600000171</v>
-      </c>
-      <c r="H27" t="s">
-        <v>88</v>
-      </c>
-      <c r="I27">
-        <v>52052192700</v>
-      </c>
-      <c r="J27" t="s">
-        <v>89</v>
-      </c>
-      <c r="K27" t="s">
-        <v>32</v>
-      </c>
       <c r="L27" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="M27" s="2">
         <v>45783</v>
@@ -2764,54 +2746,54 @@
         <v>0</v>
       </c>
       <c r="V27" t="s">
+        <v>32</v>
+      </c>
+      <c r="W27" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X27" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y27" t="s">
         <v>34</v>
-      </c>
-      <c r="W27" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X27" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y27" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
         <v>26</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D28" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E28">
         <v>2234</v>
       </c>
       <c r="F28" t="s">
-        <v>30</v>
-      </c>
-      <c r="G28">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H28" t="s">
-        <v>88</v>
-      </c>
-      <c r="I28">
-        <v>52052192700</v>
+        <v>85</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="J28" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K28" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="L28" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="M28" s="2">
         <v>45783</v>
@@ -2841,54 +2823,54 @@
         <v>0</v>
       </c>
       <c r="V28" t="s">
+        <v>32</v>
+      </c>
+      <c r="W28" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X28" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y28" t="s">
         <v>34</v>
-      </c>
-      <c r="W28" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X28" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y28" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B29" t="s">
         <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D29" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E29">
         <v>2234</v>
       </c>
       <c r="F29" t="s">
-        <v>30</v>
-      </c>
-      <c r="G29">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H29" t="s">
-        <v>88</v>
-      </c>
-      <c r="I29">
-        <v>52052192700</v>
+        <v>85</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="J29" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K29" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="L29" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="M29" s="2">
         <v>46121</v>
@@ -2918,54 +2900,54 @@
         <v>0</v>
       </c>
       <c r="V29" t="s">
+        <v>32</v>
+      </c>
+      <c r="W29" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X29" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y29" t="s">
         <v>34</v>
-      </c>
-      <c r="W29" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y29" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
         <v>26</v>
       </c>
       <c r="C30" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D30" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E30">
         <v>2234</v>
       </c>
       <c r="F30" t="s">
-        <v>30</v>
-      </c>
-      <c r="G30">
-        <v>42498600000171</v>
+        <v>85</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="H30" t="s">
-        <v>93</v>
-      </c>
-      <c r="I30">
-        <v>47913860863</v>
+        <v>85</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="J30" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="K30" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L30" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="M30" s="2">
         <v>45786</v>
@@ -2995,16 +2977,16 @@
         <v>0</v>
       </c>
       <c r="V30" t="s">
+        <v>32</v>
+      </c>
+      <c r="W30" s="2">
+        <v>46146</v>
+      </c>
+      <c r="X30" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y30" t="s">
         <v>34</v>
-      </c>
-      <c r="W30" s="2">
-        <v>46146</v>
-      </c>
-      <c r="X30" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y30" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3013,19 +2995,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TipoAtualiza_x00e7__x00e3_o xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
-    <Atualiza_x00e7__x00e3_o xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3">Só atualizar</Atualiza_x00e7__x00e3_o>
-    <GUIASREFERENTEDEPOSITOJUDICIAIS xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="a5c7d926-be96-426a-b7d8-3461508ce661" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
-    <Info xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3330,27 +3305,25 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TipoAtualiza_x00e7__x00e3_o xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
+    <Atualiza_x00e7__x00e3_o xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3">Só atualizar</Atualiza_x00e7__x00e3_o>
+    <GUIASREFERENTEDEPOSITOJUDICIAIS xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="a5c7d926-be96-426a-b7d8-3461508ce661" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
+    <Info xmlns="3787ae0c-a2f2-4ab0-991e-08818e462bd3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DECF0216-CD86-4078-B1E6-49B14E242877}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7B86-A4D3-436F-995E-125D1D1FF9CC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a5c7d926-be96-426a-b7d8-3461508ce661"/>
-    <ds:schemaRef ds:uri="3787ae0c-a2f2-4ab0-991e-08818e462bd3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3375,9 +3348,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7B86-A4D3-436F-995E-125D1D1FF9CC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DECF0216-CD86-4078-B1E6-49B14E242877}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a5c7d926-be96-426a-b7d8-3461508ce661"/>
+    <ds:schemaRef ds:uri="3787ae0c-a2f2-4ab0-991e-08818e462bd3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>